<commit_message>
test: match gwangju order spreadsheets to manual entry format
</commit_message>
<xml_diff>
--- a/test_data/gwangju_4dong_test_orders_30.xlsx
+++ b/test_data/gwangju_4dong_test_orders_30.xlsx
@@ -6,7 +6,7 @@
     <sheet name="테스트명단" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'테스트명단'!A1:H31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'테스트명단'!A1:J31</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,828 +400,1016 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:J31"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="42.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>#</v>
+      </c>
+      <c r="B1" t="str">
         <v>성명</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>전화번호</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>배송동</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>주소</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>상세주소</v>
+      </c>
+      <c r="G1" t="str">
         <v>물품내역</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>코드</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>수량</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>요청사항</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
         <v>테스트고객001</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>010-5500-1001</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>경안동</v>
       </c>
-      <c r="D2" t="str">
-        <v>경기도 광주시 경안로 10, 101동 101호</v>
-      </c>
       <c r="E2" t="str">
+        <v>경기도 광주시 경안로 10</v>
+      </c>
+      <c r="F2" t="str">
+        <v>101동 101호</v>
+      </c>
+      <c r="G2" t="str">
         <v>채소</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>T0001</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>문 앞에 놓아주세요</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
         <v>테스트고객002</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>010-5500-1002</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>송정동</v>
       </c>
-      <c r="D3" t="str">
-        <v>경기도 광주시 경안천로 110, 111동 102호</v>
-      </c>
       <c r="E3" t="str">
+        <v>경기도 광주시 경안천로 110</v>
+      </c>
+      <c r="F3" t="str">
+        <v>111동 102호</v>
+      </c>
+      <c r="G3" t="str">
         <v>과일</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>T0002</v>
       </c>
-      <c r="G3">
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>도착 전 전화 부탁드립니다</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
         <v>테스트고객003</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>010-5500-1003</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D4" t="str">
-        <v>경기도 광주시 경충대로 1407-3, 121동 103호</v>
-      </c>
       <c r="E4" t="str">
+        <v>경기도 광주시 경충대로 1407-3</v>
+      </c>
+      <c r="F4" t="str">
+        <v>121동 103호</v>
+      </c>
+      <c r="G4" t="str">
         <v>정육</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
         <v>T0003</v>
       </c>
-      <c r="G4">
+      <c r="I4">
         <v>3</v>
       </c>
-      <c r="H4" t="str">
+      <c r="J4" t="str">
         <v>천천히 오셔도 됩니다</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
         <v>테스트고객004</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>010-5500-1004</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D5" t="str">
-        <v>경기도 광주시 경안로 197, 131동 104호</v>
-      </c>
       <c r="E5" t="str">
+        <v>경기도 광주시 경안로 197</v>
+      </c>
+      <c r="F5" t="str">
+        <v>131동 104호</v>
+      </c>
+      <c r="G5" t="str">
         <v>생선</v>
       </c>
-      <c r="F5" t="str">
+      <c r="H5" t="str">
         <v>T0004</v>
       </c>
-      <c r="G5">
+      <c r="I5">
         <v>4</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <v>벨 누르지 말아주세요</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
         <v>테스트고객005</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>010-5500-1005</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>경안동</v>
       </c>
-      <c r="D6" t="str">
-        <v>경기도 광주시 경안로 104, 141동 105호</v>
-      </c>
       <c r="E6" t="str">
+        <v>경기도 광주시 경안로 104</v>
+      </c>
+      <c r="F6" t="str">
+        <v>141동 105호</v>
+      </c>
+      <c r="G6" t="str">
         <v>반찬</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>T0005</v>
       </c>
-      <c r="G6">
+      <c r="I6">
         <v>1</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <v>경비실 호출 후 전달</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
         <v>테스트고객006</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>010-5500-1006</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>송정동</v>
       </c>
-      <c r="D7" t="str">
-        <v>경기도 광주시 경안천로 113, 151동 106호</v>
-      </c>
       <c r="E7" t="str">
+        <v>경기도 광주시 경안천로 113</v>
+      </c>
+      <c r="F7" t="str">
+        <v>151동 106호</v>
+      </c>
+      <c r="G7" t="str">
         <v>쌀</v>
       </c>
-      <c r="F7" t="str">
+      <c r="H7" t="str">
         <v>T0006</v>
       </c>
-      <c r="G7">
+      <c r="I7">
         <v>2</v>
       </c>
-      <c r="H7" t="str">
+      <c r="J7" t="str">
         <v>부재 시 문고리에 걸어주세요</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
         <v>테스트고객007</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>010-5500-1007</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D8" t="str">
-        <v>경기도 광주시 경충대로 1407-5, 161동 107호</v>
-      </c>
       <c r="E8" t="str">
+        <v>경기도 광주시 경충대로 1407-5</v>
+      </c>
+      <c r="F8" t="str">
+        <v>161동 107호</v>
+      </c>
+      <c r="G8" t="str">
         <v>두부</v>
       </c>
-      <c r="F8" t="str">
+      <c r="H8" t="str">
         <v>T0007</v>
       </c>
-      <c r="G8">
+      <c r="I8">
         <v>3</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <v>문 앞에 놓아주세요</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
         <v>테스트고객008</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>010-5500-1008</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D9" t="str">
-        <v>경기도 광주시 경충대로1926번길 119, 171동 108호</v>
-      </c>
       <c r="E9" t="str">
+        <v>경기도 광주시 경충대로1926번길 119</v>
+      </c>
+      <c r="F9" t="str">
+        <v>171동 108호</v>
+      </c>
+      <c r="G9" t="str">
         <v>계란</v>
       </c>
-      <c r="F9" t="str">
+      <c r="H9" t="str">
         <v>T0008</v>
       </c>
-      <c r="G9">
+      <c r="I9">
         <v>4</v>
       </c>
-      <c r="H9" t="str">
+      <c r="J9" t="str">
         <v>도착 전 전화 부탁드립니다</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
         <v>테스트고객009</v>
       </c>
-      <c r="B10" t="str">
+      <c r="C10" t="str">
         <v>010-5500-1009</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>경안동</v>
       </c>
-      <c r="D10" t="str">
-        <v>경기도 광주시 경안로 106, 181동 109호</v>
-      </c>
       <c r="E10" t="str">
+        <v>경기도 광주시 경안로 106</v>
+      </c>
+      <c r="F10" t="str">
+        <v>181동 109호</v>
+      </c>
+      <c r="G10" t="str">
         <v>건어물</v>
       </c>
-      <c r="F10" t="str">
+      <c r="H10" t="str">
         <v>T0009</v>
       </c>
-      <c r="G10">
+      <c r="I10">
         <v>1</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <v>천천히 오셔도 됩니다</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
         <v>테스트고객010</v>
       </c>
-      <c r="B11" t="str">
+      <c r="C11" t="str">
         <v>010-5500-1010</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>송정동</v>
       </c>
-      <c r="D11" t="str">
-        <v>경기도 광주시 경안천로 114, 101동 110호</v>
-      </c>
       <c r="E11" t="str">
+        <v>경기도 광주시 경안천로 114</v>
+      </c>
+      <c r="F11" t="str">
+        <v>101동 110호</v>
+      </c>
+      <c r="G11" t="str">
         <v>생활용품</v>
       </c>
-      <c r="F11" t="str">
+      <c r="H11" t="str">
         <v>T0010</v>
       </c>
-      <c r="G11">
+      <c r="I11">
         <v>2</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <v>벨 누르지 말아주세요</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
         <v>테스트고객011</v>
       </c>
-      <c r="B12" t="str">
+      <c r="C12" t="str">
         <v>010-5500-1011</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D12" t="str">
-        <v>경기도 광주시 경충대로 1407-9, 111동 111호</v>
-      </c>
       <c r="E12" t="str">
+        <v>경기도 광주시 경충대로 1407-9</v>
+      </c>
+      <c r="F12" t="str">
+        <v>111동 111호</v>
+      </c>
+      <c r="G12" t="str">
         <v>채소</v>
       </c>
-      <c r="F12" t="str">
+      <c r="H12" t="str">
         <v>T0011</v>
       </c>
-      <c r="G12">
+      <c r="I12">
         <v>3</v>
       </c>
-      <c r="H12" t="str">
+      <c r="J12" t="str">
         <v>경비실 호출 후 전달</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
         <v>테스트고객012</v>
       </c>
-      <c r="B13" t="str">
+      <c r="C13" t="str">
         <v>010-5500-1012</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D13" t="str">
-        <v>경기도 광주시 벌원길 23, 121동 112호</v>
-      </c>
       <c r="E13" t="str">
+        <v>경기도 광주시 벌원길 23</v>
+      </c>
+      <c r="F13" t="str">
+        <v>121동 112호</v>
+      </c>
+      <c r="G13" t="str">
         <v>과일</v>
       </c>
-      <c r="F13" t="str">
+      <c r="H13" t="str">
         <v>T0012</v>
       </c>
-      <c r="G13">
+      <c r="I13">
         <v>4</v>
       </c>
-      <c r="H13" t="str">
+      <c r="J13" t="str">
         <v>부재 시 문고리에 걸어주세요</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
         <v>테스트고객013</v>
       </c>
-      <c r="B14" t="str">
+      <c r="C14" t="str">
         <v>010-5500-1013</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>경안동</v>
       </c>
-      <c r="D14" t="str">
-        <v>경기도 광주시 경안로 112, 131동 113호</v>
-      </c>
       <c r="E14" t="str">
+        <v>경기도 광주시 경안로 112</v>
+      </c>
+      <c r="F14" t="str">
+        <v>131동 113호</v>
+      </c>
+      <c r="G14" t="str">
         <v>정육</v>
       </c>
-      <c r="F14" t="str">
+      <c r="H14" t="str">
         <v>T0013</v>
       </c>
-      <c r="G14">
+      <c r="I14">
         <v>1</v>
       </c>
-      <c r="H14" t="str">
+      <c r="J14" t="str">
         <v>문 앞에 놓아주세요</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
         <v>테스트고객014</v>
       </c>
-      <c r="B15" t="str">
+      <c r="C15" t="str">
         <v>010-5500-1014</v>
       </c>
-      <c r="C15" t="str">
+      <c r="D15" t="str">
         <v>송정동</v>
       </c>
-      <c r="D15" t="str">
-        <v>경기도 광주시 경안천로 115, 141동 114호</v>
-      </c>
       <c r="E15" t="str">
+        <v>경기도 광주시 경안천로 115</v>
+      </c>
+      <c r="F15" t="str">
+        <v>141동 114호</v>
+      </c>
+      <c r="G15" t="str">
         <v>생선</v>
       </c>
-      <c r="F15" t="str">
+      <c r="H15" t="str">
         <v>T0014</v>
       </c>
-      <c r="G15">
+      <c r="I15">
         <v>2</v>
       </c>
-      <c r="H15" t="str">
+      <c r="J15" t="str">
         <v>도착 전 전화 부탁드립니다</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="str">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
         <v>테스트고객015</v>
       </c>
-      <c r="B16" t="str">
+      <c r="C16" t="str">
         <v>010-5500-1015</v>
       </c>
-      <c r="C16" t="str">
+      <c r="D16" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D16" t="str">
-        <v>경기도 광주시 경충대로 1411, 151동 115호</v>
-      </c>
       <c r="E16" t="str">
+        <v>경기도 광주시 경충대로 1411</v>
+      </c>
+      <c r="F16" t="str">
+        <v>151동 115호</v>
+      </c>
+      <c r="G16" t="str">
         <v>반찬</v>
       </c>
-      <c r="F16" t="str">
+      <c r="H16" t="str">
         <v>T0015</v>
       </c>
-      <c r="G16">
+      <c r="I16">
         <v>3</v>
       </c>
-      <c r="H16" t="str">
+      <c r="J16" t="str">
         <v>천천히 오셔도 됩니다</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="str">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
         <v>테스트고객016</v>
       </c>
-      <c r="B17" t="str">
+      <c r="C17" t="str">
         <v>010-5500-1016</v>
       </c>
-      <c r="C17" t="str">
+      <c r="D17" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D17" t="str">
-        <v>경기도 광주시 벌원길 25, 161동 116호</v>
-      </c>
       <c r="E17" t="str">
+        <v>경기도 광주시 벌원길 25</v>
+      </c>
+      <c r="F17" t="str">
+        <v>161동 116호</v>
+      </c>
+      <c r="G17" t="str">
         <v>쌀</v>
       </c>
-      <c r="F17" t="str">
+      <c r="H17" t="str">
         <v>T0016</v>
       </c>
-      <c r="G17">
+      <c r="I17">
         <v>4</v>
       </c>
-      <c r="H17" t="str">
+      <c r="J17" t="str">
         <v>벨 누르지 말아주세요</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="str">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
         <v>테스트고객017</v>
       </c>
-      <c r="B18" t="str">
+      <c r="C18" t="str">
         <v>010-5500-1017</v>
       </c>
-      <c r="C18" t="str">
+      <c r="D18" t="str">
         <v>경안동</v>
       </c>
-      <c r="D18" t="str">
-        <v>경기도 광주시 경안로 114, 171동 117호</v>
-      </c>
       <c r="E18" t="str">
+        <v>경기도 광주시 경안로 114</v>
+      </c>
+      <c r="F18" t="str">
+        <v>171동 117호</v>
+      </c>
+      <c r="G18" t="str">
         <v>두부</v>
       </c>
-      <c r="F18" t="str">
+      <c r="H18" t="str">
         <v>T0017</v>
       </c>
-      <c r="G18">
+      <c r="I18">
         <v>1</v>
       </c>
-      <c r="H18" t="str">
+      <c r="J18" t="str">
         <v>경비실 호출 후 전달</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="str">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
         <v>테스트고객018</v>
       </c>
-      <c r="B19" t="str">
+      <c r="C19" t="str">
         <v>010-5500-1018</v>
       </c>
-      <c r="C19" t="str">
+      <c r="D19" t="str">
         <v>송정동</v>
       </c>
-      <c r="D19" t="str">
-        <v>경기도 광주시 경안천로 117, 181동 118호</v>
-      </c>
       <c r="E19" t="str">
+        <v>경기도 광주시 경안천로 117</v>
+      </c>
+      <c r="F19" t="str">
+        <v>181동 118호</v>
+      </c>
+      <c r="G19" t="str">
         <v>계란</v>
       </c>
-      <c r="F19" t="str">
+      <c r="H19" t="str">
         <v>T0018</v>
       </c>
-      <c r="G19">
+      <c r="I19">
         <v>2</v>
       </c>
-      <c r="H19" t="str">
+      <c r="J19" t="str">
         <v>부재 시 문고리에 걸어주세요</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="str">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
         <v>테스트고객019</v>
       </c>
-      <c r="B20" t="str">
+      <c r="C20" t="str">
         <v>010-5500-1019</v>
       </c>
-      <c r="C20" t="str">
+      <c r="D20" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D20" t="str">
-        <v>경기도 광주시 경충대로 1413, 101동 119호</v>
-      </c>
       <c r="E20" t="str">
+        <v>경기도 광주시 경충대로 1413</v>
+      </c>
+      <c r="F20" t="str">
+        <v>101동 119호</v>
+      </c>
+      <c r="G20" t="str">
         <v>건어물</v>
       </c>
-      <c r="F20" t="str">
+      <c r="H20" t="str">
         <v>T0019</v>
       </c>
-      <c r="G20">
+      <c r="I20">
         <v>3</v>
       </c>
-      <c r="H20" t="str">
+      <c r="J20" t="str">
         <v>문 앞에 놓아주세요</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="str">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
         <v>테스트고객020</v>
       </c>
-      <c r="B21" t="str">
+      <c r="C21" t="str">
         <v>010-5500-1020</v>
       </c>
-      <c r="C21" t="str">
+      <c r="D21" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D21" t="str">
-        <v>경기도 광주시 벌원길 26, 111동 120호</v>
-      </c>
       <c r="E21" t="str">
+        <v>경기도 광주시 벌원길 26</v>
+      </c>
+      <c r="F21" t="str">
+        <v>111동 120호</v>
+      </c>
+      <c r="G21" t="str">
         <v>생활용품</v>
       </c>
-      <c r="F21" t="str">
+      <c r="H21" t="str">
         <v>T0020</v>
       </c>
-      <c r="G21">
+      <c r="I21">
         <v>4</v>
       </c>
-      <c r="H21" t="str">
+      <c r="J21" t="str">
         <v>도착 전 전화 부탁드립니다</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="str">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
         <v>테스트고객021</v>
       </c>
-      <c r="B22" t="str">
+      <c r="C22" t="str">
         <v>010-5500-1021</v>
       </c>
-      <c r="C22" t="str">
+      <c r="D22" t="str">
         <v>경안동</v>
       </c>
-      <c r="D22" t="str">
-        <v>경기도 광주시 경안로 115, 121동 101호</v>
-      </c>
       <c r="E22" t="str">
+        <v>경기도 광주시 경안로 115</v>
+      </c>
+      <c r="F22" t="str">
+        <v>121동 101호</v>
+      </c>
+      <c r="G22" t="str">
         <v>채소</v>
       </c>
-      <c r="F22" t="str">
+      <c r="H22" t="str">
         <v>T0021</v>
       </c>
-      <c r="G22">
+      <c r="I22">
         <v>1</v>
       </c>
-      <c r="H22" t="str">
+      <c r="J22" t="str">
         <v>천천히 오셔도 됩니다</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="str">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
         <v>테스트고객022</v>
       </c>
-      <c r="B23" t="str">
+      <c r="C23" t="str">
         <v>010-5500-1022</v>
       </c>
-      <c r="C23" t="str">
+      <c r="D23" t="str">
         <v>송정동</v>
       </c>
-      <c r="D23" t="str">
-        <v>경기도 광주시 경안천로 118, 131동 102호</v>
-      </c>
       <c r="E23" t="str">
+        <v>경기도 광주시 경안천로 118</v>
+      </c>
+      <c r="F23" t="str">
+        <v>131동 102호</v>
+      </c>
+      <c r="G23" t="str">
         <v>과일</v>
       </c>
-      <c r="F23" t="str">
+      <c r="H23" t="str">
         <v>T0022</v>
       </c>
-      <c r="G23">
+      <c r="I23">
         <v>2</v>
       </c>
-      <c r="H23" t="str">
+      <c r="J23" t="str">
         <v>벨 누르지 말아주세요</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="str">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
         <v>테스트고객023</v>
       </c>
-      <c r="B24" t="str">
+      <c r="C24" t="str">
         <v>010-5500-1023</v>
       </c>
-      <c r="C24" t="str">
+      <c r="D24" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D24" t="str">
-        <v>경기도 광주시 경충대로 1414, 141동 103호</v>
-      </c>
       <c r="E24" t="str">
+        <v>경기도 광주시 경충대로 1414</v>
+      </c>
+      <c r="F24" t="str">
+        <v>141동 103호</v>
+      </c>
+      <c r="G24" t="str">
         <v>정육</v>
       </c>
-      <c r="F24" t="str">
+      <c r="H24" t="str">
         <v>T0023</v>
       </c>
-      <c r="G24">
+      <c r="I24">
         <v>3</v>
       </c>
-      <c r="H24" t="str">
+      <c r="J24" t="str">
         <v>경비실 호출 후 전달</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="str">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
         <v>테스트고객024</v>
       </c>
-      <c r="B25" t="str">
+      <c r="C25" t="str">
         <v>010-5500-1024</v>
       </c>
-      <c r="C25" t="str">
+      <c r="D25" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D25" t="str">
-        <v>경기도 광주시 벌원길 34, 151동 104호</v>
-      </c>
       <c r="E25" t="str">
+        <v>경기도 광주시 벌원길 34</v>
+      </c>
+      <c r="F25" t="str">
+        <v>151동 104호</v>
+      </c>
+      <c r="G25" t="str">
         <v>생선</v>
       </c>
-      <c r="F25" t="str">
+      <c r="H25" t="str">
         <v>T0024</v>
       </c>
-      <c r="G25">
+      <c r="I25">
         <v>4</v>
       </c>
-      <c r="H25" t="str">
+      <c r="J25" t="str">
         <v>부재 시 문고리에 걸어주세요</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="str">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
         <v>테스트고객025</v>
       </c>
-      <c r="B26" t="str">
+      <c r="C26" t="str">
         <v>010-5500-1025</v>
       </c>
-      <c r="C26" t="str">
+      <c r="D26" t="str">
         <v>경안동</v>
       </c>
-      <c r="D26" t="str">
-        <v>경기도 광주시 경안로 116, 161동 105호</v>
-      </c>
       <c r="E26" t="str">
+        <v>경기도 광주시 경안로 116</v>
+      </c>
+      <c r="F26" t="str">
+        <v>161동 105호</v>
+      </c>
+      <c r="G26" t="str">
         <v>반찬</v>
       </c>
-      <c r="F26" t="str">
+      <c r="H26" t="str">
         <v>T0025</v>
       </c>
-      <c r="G26">
+      <c r="I26">
         <v>1</v>
       </c>
-      <c r="H26" t="str">
+      <c r="J26" t="str">
         <v>문 앞에 놓아주세요</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="str">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
         <v>테스트고객026</v>
       </c>
-      <c r="B27" t="str">
+      <c r="C27" t="str">
         <v>010-5500-1026</v>
       </c>
-      <c r="C27" t="str">
+      <c r="D27" t="str">
         <v>송정동</v>
       </c>
-      <c r="D27" t="str">
-        <v>경기도 광주시 경안천로 119, 171동 106호</v>
-      </c>
       <c r="E27" t="str">
+        <v>경기도 광주시 경안천로 119</v>
+      </c>
+      <c r="F27" t="str">
+        <v>171동 106호</v>
+      </c>
+      <c r="G27" t="str">
         <v>쌀</v>
       </c>
-      <c r="F27" t="str">
+      <c r="H27" t="str">
         <v>T0026</v>
       </c>
-      <c r="G27">
+      <c r="I27">
         <v>2</v>
       </c>
-      <c r="H27" t="str">
+      <c r="J27" t="str">
         <v>도착 전 전화 부탁드립니다</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="str">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
         <v>테스트고객027</v>
       </c>
-      <c r="B28" t="str">
+      <c r="C28" t="str">
         <v>010-5500-1027</v>
       </c>
-      <c r="C28" t="str">
+      <c r="D28" t="str">
         <v>쌍령동</v>
       </c>
-      <c r="D28" t="str">
-        <v>경기도 광주시 경충대로 1425, 181동 107호</v>
-      </c>
       <c r="E28" t="str">
+        <v>경기도 광주시 경충대로 1425</v>
+      </c>
+      <c r="F28" t="str">
+        <v>181동 107호</v>
+      </c>
+      <c r="G28" t="str">
         <v>두부</v>
       </c>
-      <c r="F28" t="str">
+      <c r="H28" t="str">
         <v>T0027</v>
       </c>
-      <c r="G28">
+      <c r="I28">
         <v>3</v>
       </c>
-      <c r="H28" t="str">
+      <c r="J28" t="str">
         <v>천천히 오셔도 됩니다</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="str">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
         <v>테스트고객028</v>
       </c>
-      <c r="B29" t="str">
+      <c r="C29" t="str">
         <v>010-5500-1028</v>
       </c>
-      <c r="C29" t="str">
+      <c r="D29" t="str">
         <v>탄벌동</v>
       </c>
-      <c r="D29" t="str">
-        <v>경기도 광주시 벌원길 36, 101동 108호</v>
-      </c>
       <c r="E29" t="str">
+        <v>경기도 광주시 벌원길 36</v>
+      </c>
+      <c r="F29" t="str">
+        <v>101동 108호</v>
+      </c>
+      <c r="G29" t="str">
         <v>계란</v>
       </c>
-      <c r="F29" t="str">
+      <c r="H29" t="str">
         <v>T0028</v>
       </c>
-      <c r="G29">
+      <c r="I29">
         <v>4</v>
       </c>
-      <c r="H29" t="str">
+      <c r="J29" t="str">
         <v>벨 누르지 말아주세요</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="str">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
         <v>테스트고객029</v>
       </c>
-      <c r="B30" t="str">
+      <c r="C30" t="str">
         <v>010-5500-1029</v>
       </c>
-      <c r="C30" t="str">
+      <c r="D30" t="str">
         <v>경안동</v>
       </c>
-      <c r="D30" t="str">
-        <v>경기도 광주시 경안로 117, 111동 109호</v>
-      </c>
       <c r="E30" t="str">
+        <v>경기도 광주시 경안로 117</v>
+      </c>
+      <c r="F30" t="str">
+        <v>111동 109호</v>
+      </c>
+      <c r="G30" t="str">
         <v>건어물</v>
       </c>
-      <c r="F30" t="str">
+      <c r="H30" t="str">
         <v>T0029</v>
       </c>
-      <c r="G30">
+      <c r="I30">
         <v>1</v>
       </c>
-      <c r="H30" t="str">
+      <c r="J30" t="str">
         <v>경비실 호출 후 전달</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="str">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
         <v>테스트고객030</v>
       </c>
-      <c r="B31" t="str">
+      <c r="C31" t="str">
         <v>010-5500-1030</v>
       </c>
-      <c r="C31" t="str">
+      <c r="D31" t="str">
         <v>송정동</v>
       </c>
-      <c r="D31" t="str">
-        <v>경기도 광주시 경안천로 121, 121동 110호</v>
-      </c>
       <c r="E31" t="str">
+        <v>경기도 광주시 경안천로 121</v>
+      </c>
+      <c r="F31" t="str">
+        <v>121동 110호</v>
+      </c>
+      <c r="G31" t="str">
         <v>생활용품</v>
       </c>
-      <c r="F31" t="str">
+      <c r="H31" t="str">
         <v>T0030</v>
       </c>
-      <c r="G31">
+      <c r="I31">
         <v>2</v>
       </c>
-      <c r="H31" t="str">
+      <c r="J31" t="str">
         <v>부재 시 문고리에 걸어주세요</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:J31"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>